<commit_message>
Macro hasta 3G BB Ok
</commit_message>
<xml_diff>
--- a/Macro_4G_Streamlit/LA781 - TEKNICA/LA781 - TEKNICA/RND_ULA781_WCDMA1900_900_20251104-141953.xlsx
+++ b/Macro_4G_Streamlit/LA781 - TEKNICA/LA781 - TEKNICA/RND_ULA781_WCDMA1900_900_20251104-141953.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
-  <workbookPr defaultThemeVersion="202300"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://olitelltda-my.sharepoint.com/personal/jcavieres_olitel_cl/Documents/000_Shared_Integracion/2025/RAN/011-Noviembre/LA781 - TEKNICA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pledesma\Documents\Piero Ledesma\Piero Ledesma\Nuevas Macros\Macro_4G_Streamlit\LA781 - TEKNICA\LA781 - TEKNICA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{EA6ECAE6-247D-4E56-ABBE-43346E1D8D50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0564F22-644A-46E9-8846-9B654C41BA28}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="758" firstSheet="17" activeTab="30" xr2:uid="{F2C12E03-F76D-4453-AA91-2AB7B814A7C4}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13275" windowHeight="6360" tabRatio="758" firstSheet="12" activeTab="19"/>
   </bookViews>
   <sheets>
     <sheet name="EUL" sheetId="32" r:id="rId1"/>
@@ -73,7 +72,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">UtranCell!$A$1:$GQ$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">UtranRelation!$A$1:$L$123</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -94,7 +93,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2340" uniqueCount="710">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2340" uniqueCount="711">
   <si>
     <t>Pop</t>
   </si>
@@ -2224,12 +2223,15 @@
   </si>
   <si>
     <t>RUS01 B8</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> y " </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="8">
     <font>
       <sz val="11"/>
@@ -2414,10 +2416,10 @@
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 172" xfId="2" xr:uid="{B4E57848-AABA-4490-B5BE-58621C32CD11}"/>
-    <cellStyle name="Normal 175" xfId="1" xr:uid="{43F51F44-458A-46C5-B88E-39EFB96C7849}"/>
-    <cellStyle name="Normal 2 10" xfId="4" xr:uid="{2C723194-41AC-4BB4-81F9-F7AED4D0E465}"/>
-    <cellStyle name="Normal 6 2" xfId="3" xr:uid="{33F635B6-B831-4493-9236-CE5F35464047}"/>
+    <cellStyle name="Normal 172" xfId="2"/>
+    <cellStyle name="Normal 175" xfId="1"/>
+    <cellStyle name="Normal 2 10" xfId="4"/>
+    <cellStyle name="Normal 6 2" xfId="3"/>
   </cellStyles>
   <dxfs count="3">
     <dxf>
@@ -2779,26 +2781,26 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEA72F82-C089-470E-8E54-39EA656AC547}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:U7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.125" bestFit="1" customWidth="1"/>
     <col min="4" max="8" width="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="3.875" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="4.875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="4.375" bestFit="1" customWidth="1"/>
     <col min="15" max="18" width="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="3.875" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="3.42578125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="3.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="5" customFormat="1" ht="156">
+    <row r="1" spans="1:21" s="5" customFormat="1" ht="156.75">
       <c r="A1" s="12" t="s">
         <v>23</v>
       </c>
@@ -3241,20 +3243,20 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D22AC29-5AEB-4340-A633-36F4F7FFB1C3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
   </sheetPr>
   <dimension ref="A1:K19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.375" bestFit="1" customWidth="1"/>
     <col min="2" max="4" width="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="37.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="37.625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="37.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="114.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="37.625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="114.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="5" customFormat="1" ht="85.5">
@@ -3900,25 +3902,26 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{740A98FE-509D-4102-802C-19C950029B81}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.375" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="55.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="3.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="55.375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3.875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.125" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="5" customFormat="1" ht="132">
+    <row r="1" spans="1:10" s="5" customFormat="1" ht="133.5">
       <c r="A1" s="12" t="s">
         <v>23</v>
       </c>
@@ -3988,24 +3991,24 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BD12399-7394-471A-B17D-F3145190FA3F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:W2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="3.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.875" bestFit="1" customWidth="1"/>
     <col min="5" max="7" width="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="3.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="12" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="3.875" bestFit="1" customWidth="1"/>
+    <col min="9" max="12" width="4.875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="23.875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="3.875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="5" customFormat="1" ht="126.75">
+    <row r="1" spans="1:23" s="5" customFormat="1" ht="128.25">
       <c r="A1" s="23" t="s">
         <v>23</v>
       </c>
@@ -4123,21 +4126,21 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C24EF348-4C2A-4E03-B42A-F2A0C4C791A8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
   </sheetPr>
   <dimension ref="A1:O1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.375" bestFit="1" customWidth="1"/>
     <col min="2" max="5" width="3" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="12" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="9.125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="3.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="5" customFormat="1" ht="173.25">
+    <row r="1" spans="1:15" s="5" customFormat="1" ht="174">
       <c r="A1" s="10" t="s">
         <v>61</v>
       </c>
@@ -4180,21 +4183,21 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B932F145-C02A-437C-9825-162895D4EA76}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
   </sheetPr>
   <dimension ref="A1:K1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.375" bestFit="1" customWidth="1"/>
     <col min="2" max="4" width="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="3.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="3.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="3.875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3.125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="5" customFormat="1" ht="96">
+    <row r="1" spans="1:11" s="5" customFormat="1" ht="96.75">
       <c r="A1" s="10" t="s">
         <v>61</v>
       </c>
@@ -4227,43 +4230,43 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54D7EFC9-85ED-4F32-B181-2A742A5994A9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
   </sheetPr>
   <dimension ref="A1:BW7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.375" bestFit="1" customWidth="1"/>
     <col min="4" max="11" width="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="4.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="4.375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="3.875" bestFit="1" customWidth="1"/>
     <col min="14" max="19" width="3" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="3.875" bestFit="1" customWidth="1"/>
     <col min="21" max="31" width="3" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="3.42578125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="4.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="3.85546875" bestFit="1" customWidth="1"/>
-    <col min="36" max="37" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="3.375" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="4.375" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="5.875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="3.875" bestFit="1" customWidth="1"/>
+    <col min="36" max="37" width="4.375" bestFit="1" customWidth="1"/>
     <col min="38" max="40" width="3" bestFit="1" customWidth="1"/>
-    <col min="41" max="42" width="4.42578125" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="34.140625" bestFit="1" customWidth="1"/>
+    <col min="41" max="42" width="4.375" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="34.125" bestFit="1" customWidth="1"/>
     <col min="44" max="44" width="3" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="3.875" bestFit="1" customWidth="1"/>
     <col min="46" max="46" width="3" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="3.875" bestFit="1" customWidth="1"/>
     <col min="48" max="53" width="3" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="40.140625" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="40.125" bestFit="1" customWidth="1"/>
     <col min="55" max="59" width="3" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="43.140625" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="43.125" bestFit="1" customWidth="1"/>
     <col min="61" max="73" width="3" bestFit="1" customWidth="1"/>
-    <col min="74" max="75" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="74" max="75" width="4.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:75" s="5" customFormat="1" ht="171">
+    <row r="1" spans="1:75" s="5" customFormat="1" ht="171.75">
       <c r="A1" s="10" t="s">
         <v>23</v>
       </c>
@@ -5810,20 +5813,20 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1E851C7-8B42-4351-A82A-47F891CC2CAA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
   </sheetPr>
   <dimension ref="A1:M22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.125" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="3.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="3.875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="15.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="5" customFormat="1" ht="119.25">
@@ -5972,7 +5975,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>269</v>
+        <v>710</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>265</v>
@@ -6554,26 +6557,27 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49A1A5D2-AE98-4C38-9B40-7664934FDFF9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:T7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="3.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="3.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="19" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="3.875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3.875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.375" bestFit="1" customWidth="1"/>
+    <col min="8" max="19" width="8.375" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="5" customFormat="1" ht="51">
+    <row r="1" spans="1:20" s="5" customFormat="1" ht="51.75">
       <c r="A1" s="12" t="s">
         <v>23</v>
       </c>
@@ -7013,14 +7017,14 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{286DA3A7-FA5F-4444-99B2-03806C4A3E94}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="5" customFormat="1" ht="26.25">
@@ -7073,16 +7077,16 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07088852-566F-4B16-8619-F538EEA54714}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="3.875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7152,13 +7156,13 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E3510D6-7BB4-4B1D-9C4B-C4ADB3157612}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.125" bestFit="1" customWidth="1"/>
     <col min="4" max="9" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7392,19 +7396,19 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCFFA804-0DE0-45EC-8B7B-7E03B206B52C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L123"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.125" bestFit="1" customWidth="1"/>
     <col min="6" max="8" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="5" customFormat="1" ht="75">
+    <row r="1" spans="1:12" s="5" customFormat="1" ht="75.75">
       <c r="A1" s="4" t="s">
         <v>182</v>
       </c>
@@ -11098,20 +11102,20 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEF00701-C710-45C5-BC8D-3D969175C3EC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="7.125" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3.875" bestFit="1" customWidth="1"/>
     <col min="7" max="9" width="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="5" customFormat="1" ht="156.75">
+    <row r="1" spans="1:12" s="5" customFormat="1" ht="157.5">
       <c r="A1" s="12" t="s">
         <v>23</v>
       </c>
@@ -11369,22 +11373,22 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE92FEAD-89C0-4F2B-AD27-D9DE23454488}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L31"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.375" bestFit="1" customWidth="1"/>
     <col min="6" max="8" width="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="5" customFormat="1" ht="102.75">
+    <row r="1" spans="1:12" s="5" customFormat="1" ht="103.5">
       <c r="A1" s="12" t="s">
         <v>23</v>
       </c>
@@ -12506,14 +12510,14 @@
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8950BFA3-7044-4C32-B5C7-C130F07D3664}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="6" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="5" customFormat="1" ht="96">
+    <row r="1" spans="1:6" s="5" customFormat="1" ht="96.75">
       <c r="A1" s="12" t="s">
         <v>23</v>
       </c>
@@ -12539,14 +12543,14 @@
 </file>
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C932DB1A-C2CC-42DC-ACED-4E58CF204BFA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="8" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="5" customFormat="1" ht="71.25">
+    <row r="1" spans="1:8" s="5" customFormat="1" ht="72">
       <c r="A1" s="12" t="s">
         <v>151</v>
       </c>
@@ -12578,14 +12582,14 @@
 </file>
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF965CAB-18E1-40B4-8597-16576AE0028B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="3" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="5" customFormat="1" ht="61.5">
+    <row r="1" spans="1:6" s="5" customFormat="1" ht="62.25">
       <c r="A1" s="12" t="s">
         <v>148</v>
       </c>
@@ -12605,14 +12609,14 @@
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{410BE0B5-E0E8-4686-98F2-387465782F4F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="2" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="5" customFormat="1" ht="56.25">
+    <row r="1" spans="1:12" s="5" customFormat="1" ht="57">
       <c r="A1" s="12" t="s">
         <v>146</v>
       </c>
@@ -12650,24 +12654,24 @@
 </file>
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F55D754-050A-45EB-8547-CD0818127247}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:S7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.375" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="3.875" bestFit="1" customWidth="1"/>
     <col min="10" max="17" width="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="17.625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="7.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="5" customFormat="1" ht="144.75">
+    <row r="1" spans="1:19" s="5" customFormat="1" ht="145.5">
       <c r="A1" s="12" t="s">
         <v>126</v>
       </c>
@@ -13086,19 +13090,19 @@
 </file>
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE857EAE-323B-4748-8EC8-7A31838FE2C6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
   </sheetPr>
   <dimension ref="A1:BN2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.375" bestFit="1" customWidth="1"/>
     <col min="3" max="66" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:66" s="5" customFormat="1" ht="145.5">
+    <row r="1" spans="1:66" s="5" customFormat="1" ht="146.25">
       <c r="A1" s="10" t="s">
         <v>23</v>
       </c>
@@ -13509,21 +13513,22 @@
     <cfRule type="duplicateValues" dxfId="0" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49766CBD-DA1F-448B-B893-F4AA005F5B3C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.25" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="3.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3.875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="5" customFormat="1" ht="94.5">
@@ -13812,19 +13817,19 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E949E76-6EC0-45FD-AE39-7E837A3F8178}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:X7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.125" bestFit="1" customWidth="1"/>
     <col min="4" max="17" width="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="3.875" bestFit="1" customWidth="1"/>
     <col min="19" max="24" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="5" customFormat="1" ht="141">
+    <row r="1" spans="1:24" s="5" customFormat="1" ht="141.75">
       <c r="A1" s="12" t="s">
         <v>23</v>
       </c>
@@ -14264,19 +14269,19 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30421453-DC46-467F-A0A4-14CC0C44A89F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:P25"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="59.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="59.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="5" customFormat="1" ht="99.75">
+    <row r="1" spans="1:16" s="5" customFormat="1" ht="100.5">
       <c r="A1" s="4" t="s">
         <v>23</v>
       </c>
@@ -15032,24 +15037,24 @@
 </file>
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5527FC4-35B5-4D87-ACE4-CA1E91E5B689}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:P7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="3.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="3.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="3.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="3.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3.125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="3.875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="3.125" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="7.125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="5" customFormat="1" ht="77.25">
+    <row r="1" spans="1:16" s="5" customFormat="1" ht="78">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -15363,13 +15368,13 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8D47E83-2A70-463D-A1C3-26C48FF765D5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.125" bestFit="1" customWidth="1"/>
     <col min="4" max="7" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -15575,23 +15580,23 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1583F90-B5CF-46AE-A4FF-AF7E98A8041D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:R7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.125" bestFit="1" customWidth="1"/>
     <col min="4" max="6" width="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="3.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="3.375" bestFit="1" customWidth="1"/>
     <col min="8" max="12" width="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.875" bestFit="1" customWidth="1"/>
     <col min="14" max="15" width="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="4.875" bestFit="1" customWidth="1"/>
     <col min="17" max="18" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="5" customFormat="1" ht="147">
+    <row r="1" spans="1:18" s="5" customFormat="1" ht="147.75">
       <c r="A1" s="12" t="s">
         <v>23</v>
       </c>
@@ -15989,15 +15994,15 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E22D1C9-8D8E-42FF-8C41-13BB918A8916}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Q7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.125" bestFit="1" customWidth="1"/>
     <col min="4" max="10" width="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="3.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="3.375" bestFit="1" customWidth="1"/>
     <col min="12" max="17" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -16354,94 +16359,94 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{120A74AF-A7CD-4A7F-9C72-93E7E734A46E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:GQ58"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.125" bestFit="1" customWidth="1"/>
     <col min="4" max="8" width="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="23.875" bestFit="1" customWidth="1"/>
     <col min="12" max="16" width="3" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="5.875" bestFit="1" customWidth="1"/>
     <col min="19" max="21" width="3" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.875" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="3" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="25" max="31" width="3.85546875" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="3.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="25" max="31" width="3.875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="3.375" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="3" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="5.875" bestFit="1" customWidth="1"/>
     <col min="35" max="35" width="3" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="5.875" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="3.875" bestFit="1" customWidth="1"/>
     <col min="38" max="40" width="3" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="3.875" bestFit="1" customWidth="1"/>
     <col min="42" max="51" width="3" bestFit="1" customWidth="1"/>
-    <col min="52" max="54" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="52" max="54" width="3.875" bestFit="1" customWidth="1"/>
     <col min="55" max="57" width="3" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="3.875" bestFit="1" customWidth="1"/>
     <col min="59" max="66" width="3" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="4.375" bestFit="1" customWidth="1"/>
     <col min="68" max="71" width="3" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="3.875" bestFit="1" customWidth="1"/>
     <col min="73" max="77" width="3" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="3.875" bestFit="1" customWidth="1"/>
     <col min="79" max="85" width="3" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="3.85546875" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="88" max="88" width="3.42578125" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="3.875" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="4.875" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="3.375" bestFit="1" customWidth="1"/>
     <col min="89" max="97" width="3" bestFit="1" customWidth="1"/>
-    <col min="98" max="98" width="3.85546875" bestFit="1" customWidth="1"/>
-    <col min="99" max="99" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="100" max="100" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="98" max="98" width="3.875" bestFit="1" customWidth="1"/>
+    <col min="99" max="99" width="17.75" bestFit="1" customWidth="1"/>
+    <col min="100" max="100" width="5.875" bestFit="1" customWidth="1"/>
     <col min="101" max="102" width="3" bestFit="1" customWidth="1"/>
-    <col min="103" max="103" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="103" max="103" width="3.875" bestFit="1" customWidth="1"/>
     <col min="104" max="105" width="3" bestFit="1" customWidth="1"/>
-    <col min="106" max="106" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="107" max="107" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="106" max="106" width="5.875" bestFit="1" customWidth="1"/>
+    <col min="107" max="107" width="3.875" bestFit="1" customWidth="1"/>
     <col min="108" max="108" width="3" bestFit="1" customWidth="1"/>
-    <col min="109" max="109" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="109" max="109" width="5.875" bestFit="1" customWidth="1"/>
     <col min="110" max="110" width="3" bestFit="1" customWidth="1"/>
-    <col min="111" max="111" width="3.85546875" bestFit="1" customWidth="1"/>
-    <col min="112" max="112" width="3.42578125" bestFit="1" customWidth="1"/>
-    <col min="113" max="113" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="111" max="111" width="3.875" bestFit="1" customWidth="1"/>
+    <col min="112" max="112" width="3.375" bestFit="1" customWidth="1"/>
+    <col min="113" max="113" width="4.375" bestFit="1" customWidth="1"/>
     <col min="114" max="114" width="3" bestFit="1" customWidth="1"/>
-    <col min="115" max="115" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="115" max="115" width="22.375" bestFit="1" customWidth="1"/>
     <col min="116" max="117" width="3" bestFit="1" customWidth="1"/>
-    <col min="118" max="119" width="3.85546875" bestFit="1" customWidth="1"/>
-    <col min="120" max="120" width="3.42578125" bestFit="1" customWidth="1"/>
-    <col min="121" max="121" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="118" max="119" width="3.875" bestFit="1" customWidth="1"/>
+    <col min="120" max="120" width="3.375" bestFit="1" customWidth="1"/>
+    <col min="121" max="121" width="3.875" bestFit="1" customWidth="1"/>
     <col min="122" max="122" width="3" bestFit="1" customWidth="1"/>
-    <col min="123" max="127" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="123" max="127" width="3.875" bestFit="1" customWidth="1"/>
     <col min="128" max="129" width="3" bestFit="1" customWidth="1"/>
-    <col min="130" max="130" width="3.42578125" bestFit="1" customWidth="1"/>
-    <col min="131" max="131" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="130" max="130" width="3.375" bestFit="1" customWidth="1"/>
+    <col min="131" max="131" width="4.375" bestFit="1" customWidth="1"/>
     <col min="132" max="132" width="3" bestFit="1" customWidth="1"/>
-    <col min="133" max="133" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="133" max="133" width="3.875" bestFit="1" customWidth="1"/>
     <col min="134" max="149" width="3" bestFit="1" customWidth="1"/>
-    <col min="150" max="150" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="150" max="150" width="5.875" bestFit="1" customWidth="1"/>
     <col min="151" max="151" width="3" bestFit="1" customWidth="1"/>
-    <col min="152" max="152" width="3.42578125" bestFit="1" customWidth="1"/>
+    <col min="152" max="152" width="3.375" bestFit="1" customWidth="1"/>
     <col min="153" max="154" width="3" bestFit="1" customWidth="1"/>
-    <col min="155" max="155" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="155" max="155" width="3.875" bestFit="1" customWidth="1"/>
     <col min="156" max="160" width="3" bestFit="1" customWidth="1"/>
-    <col min="161" max="161" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="161" max="161" width="3.875" bestFit="1" customWidth="1"/>
     <col min="162" max="169" width="3" bestFit="1" customWidth="1"/>
-    <col min="170" max="170" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="170" max="170" width="14.875" bestFit="1" customWidth="1"/>
     <col min="171" max="178" width="3" bestFit="1" customWidth="1"/>
-    <col min="179" max="180" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="181" max="181" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="182" max="182" width="3.42578125" bestFit="1" customWidth="1"/>
-    <col min="183" max="183" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="179" max="180" width="4.875" bestFit="1" customWidth="1"/>
+    <col min="181" max="181" width="11.25" bestFit="1" customWidth="1"/>
+    <col min="182" max="182" width="3.375" bestFit="1" customWidth="1"/>
+    <col min="183" max="183" width="4.375" bestFit="1" customWidth="1"/>
     <col min="184" max="194" width="3" bestFit="1" customWidth="1"/>
-    <col min="195" max="195" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="195" max="195" width="7.125" bestFit="1" customWidth="1"/>
     <col min="196" max="198" width="3" bestFit="1" customWidth="1"/>
-    <col min="199" max="199" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="199" max="199" width="19.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:199" s="5" customFormat="1" ht="237">
+    <row r="1" spans="1:199" s="5" customFormat="1" ht="238.5">
       <c r="A1" s="23" t="s">
         <v>23</v>
       </c>
@@ -30855,17 +30860,17 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{115C8CF1-D1EE-430A-BE3F-2B3924A81F97}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
   </sheetPr>
   <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="3" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="5" customFormat="1" ht="104.25">
+    <row r="1" spans="1:3" s="5" customFormat="1" ht="105">
       <c r="A1" s="21" t="s">
         <v>61</v>
       </c>
@@ -30882,35 +30887,35 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E90D853C-7384-47DC-A1A5-AEB65F3638FD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
   </sheetPr>
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.875" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="3.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="4.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="3.875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.375" bestFit="1" customWidth="1"/>
     <col min="12" max="13" width="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="3.875" bestFit="1" customWidth="1"/>
     <col min="16" max="20" width="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="3.85546875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="3.875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="5.875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="4.875" bestFit="1" customWidth="1"/>
     <col min="24" max="25" width="3" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="12.375" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="5" customFormat="1" ht="106.5">
+    <row r="1" spans="1:28" s="5" customFormat="1" ht="107.25">
       <c r="A1" s="21" t="s">
         <v>23</v>
       </c>

</xml_diff>